<commit_message>
changed to user based permission
</commit_message>
<xml_diff>
--- a/backend/users.xlsx
+++ b/backend/users.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,21 @@
           <t>role</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -471,21 +486,28 @@
           <t>analyst</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>a88dbb9c5e67</t>
+          <t>8dd9a8e73e32</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>farmer1@gmail.com</t>
+          <t>farmer3@gmail.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>scrypt:32768:8:1$Et5o8WNrDcirUibo$06e84719eb08781af6c7992c7e774e9aeb3825de76bce15cef7b6f628b7806ceede0314c67ffc35bab6ec286da3658906d4aa29386d3d3bc2207c33a9375c79a</t>
+          <t>271002</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -493,104 +515,139 @@
           <t>farmer</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>5842e0942a5c</t>
+          <t>18ff9913c5aa</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>farmer2@gmail.com</t>
+          <t>debdeep.guha@gmail.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>scrypt:32768:8:1$vYIk4Ghll677RxA8$f7751d2f21c4c981e14e41265078db5ff3292740fd60e90e924e759bd0f5324e95332890f84b008b537c77188b08f8612bb5699e5bf50777949986c0dc011191</t>
+          <t>112233</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>farmer</t>
-        </is>
-      </c>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8dd9a8e73e32</t>
+          <t>c1019934ab0f</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>farmer3@gmail.com</t>
+          <t>snigdho@gmail.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>271002</t>
+          <t>123456</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>farmer</t>
-        </is>
-      </c>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18ff9913c5aa</t>
+          <t>28f2311068bf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>debdeep.guha@gmail.com</t>
+          <t>farmer4@gmail.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>112233</t>
+          <t>123456</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>admin</t>
-        </is>
-      </c>
+          <t>farmer</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>c1019934ab0f</t>
+          <t>ea0740f07543</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>snigdho@gmail.com</t>
+          <t>tuteck@gmail.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>123456</t>
+          <t>112233</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>analyst</t>
-        </is>
-      </c>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>28f2311068bf</t>
+          <t>7e99f2f642cf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>farmer4@gmail.com</t>
+          <t>tuteck2@gmail.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -600,19 +657,26 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>farmer</t>
-        </is>
-      </c>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ea0740f07543</t>
+          <t>51bbcd801705</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>tuteck@gmail.com</t>
+          <t>state_admin_rajasthan@gmail.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -622,29 +686,55 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>admin</t>
-        </is>
-      </c>
+          <t>state_admin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>rajasthan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7e99f2f642cf</t>
+          <t>825c2c026597</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>tuteck2@gmail.com</t>
+          <t>district_admin_ajmer@gmail.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>123456</t>
+          <t>112233</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>analyst</t>
+          <t>district_admin</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>rajasthan</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Ajmer</t>
         </is>
       </c>
     </row>

</xml_diff>